<commit_message>
commit catdriver bug fix
</commit_message>
<xml_diff>
--- a/modules/tabs/docs/templates/Survey_Structure_Template.xlsx
+++ b/modules/tabs/docs/templates/Survey_Structure_Template.xlsx
@@ -1,43 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duncan/Documents/Turas/modules/tabs/docs/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A10841D-23E9-B142-A551-06F014645324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="23380" windowHeight="24000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23380" windowHeight="24000" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
-    <sheet name="Project" sheetId="5" r:id="rId2"/>
-    <sheet name="Questions" sheetId="2" r:id="rId3"/>
-    <sheet name="Options" sheetId="3" r:id="rId4"/>
-    <sheet name="Composite_Metrics" sheetId="4" r:id="rId5"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Project" sheetId="5" state="visible" r:id="rId2"/>
+    <sheet name="Questions" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Options" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Composite_Metrics" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
   <si>
     <t>Survey Structure Template - Instructions</t>
   </si>
@@ -1160,7 +1140,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,44 +1150,44 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <b/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF366092"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="16"/>
       <color rgb="FF366092"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b/>
     </font>
     <font>
-      <i/>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <i/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF366092"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b/>
     </font>
     <font>
       <sz val="12"/>
@@ -1221,34 +1202,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
     </font>
     <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri (Body)"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1292,7 +1260,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -1304,27 +1271,26 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1333,8 +1299,23 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1342,31 +1323,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{EF8A5AE8-860E-9343-9C01-5902C3C53574}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1665,173 +1627,173 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="80" customWidth="1"/>
+    <col min="1" max="1" width="80" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-    </row>
-    <row r="4" spans="1:6" ht="19" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="4" ht="19" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+    <row r="5">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-    </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="24" t="s">
+    <row r="10">
+      <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="24" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="24" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="24" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="24" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-    </row>
-    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="24" t="s">
+    <row r="17">
+      <c r="A17" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="24" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="24" t="s">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="24" t="s">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="24" t="s">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1850,312 +1812,314 @@
     <mergeCell ref="A13:F13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{497186D7-97EC-4E4F-B22C-9EE5EDDDB3C3}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="24.83203125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="36.1640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="9.5" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="80.83203125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1">
+      <c r="A1" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3">
+      <c r="A3" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+    <row r="4">
+      <c r="A4" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="9" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+    <row r="5">
+      <c r="A5" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="8"/>
+      <c r="C5" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    <row r="6">
+      <c r="A6" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7">
+      <c r="A7" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="8" t="n">
         <v>20251018</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+    <row r="8">
+      <c r="A8" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+    <row r="9">
+      <c r="A9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="9" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+    <row r="10">
+      <c r="A10" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="5" t="s">
+      <c r="B10" s="8"/>
+      <c r="C10" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+    <row r="11">
+      <c r="A11" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="5" t="s">
+      <c r="B11" s="8"/>
+      <c r="C11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    <row r="12">
+      <c r="A12" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="5" t="s">
+      <c r="B12" s="8"/>
+      <c r="C12" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+    <row r="13">
+      <c r="A13" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+    <row r="14">
+      <c r="A14" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="5" t="s">
+      <c r="B14" s="8"/>
+      <c r="C14" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+    <row r="15">
+      <c r="A15" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="5" t="s">
+      <c r="B15" s="8"/>
+      <c r="C15" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="9" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+    <row r="16">
+      <c r="A16" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="9" t="s">
         <v>71</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="12.33203125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1">
+      <c r="A1" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-    </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="9"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-    </row>
-    <row r="4" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="20"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="20"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
@@ -2168,45 +2132,45 @@
       <c r="K4" s="10"/>
       <c r="L4" s="10"/>
     </row>
-    <row r="5" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+    <row r="5" ht="68" customHeight="1">
       <c r="A5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="I5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="J5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="L5" s="14" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="187" x14ac:dyDescent="0.2">
+    <row r="6" ht="187" customHeight="1">
       <c r="A6" s="12" t="s">
         <v>19</v>
       </c>
@@ -2244,7 +2208,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" ht="51" customHeight="1">
       <c r="A7" s="12" t="s">
         <v>37</v>
       </c>
@@ -2282,7 +2246,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="12" t="s">
         <v>77</v>
       </c>
@@ -2293,13 +2257,13 @@
         <v>98</v>
       </c>
       <c r="D8" s="13"/>
-      <c r="E8" s="13">
+      <c r="E8" s="13" t="n">
         <v>5</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="13" t="n">
         <v>3</v>
       </c>
       <c r="H8" s="13" t="s">
@@ -2311,277 +2275,285 @@
       <c r="J8" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="13">
+      <c r="L8" s="13" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="19" t="s">
+    <row r="12">
+      <c r="A12" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-    </row>
-    <row r="13" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-    </row>
-    <row r="14" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="18" t="s">
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-    </row>
-    <row r="15" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-    </row>
-    <row r="16" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="18" t="s">
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-    </row>
-    <row r="17" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="18" t="s">
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-    </row>
-    <row r="18" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="18" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-    </row>
-    <row r="19" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="18" t="s">
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-    </row>
-    <row r="20" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="18" t="s">
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-    </row>
-    <row r="22" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B22" s="9" t="s">
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="20" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B23" s="9" t="s">
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="20" t="s">
         <v>178</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="9" width="14.1640625" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" customWidth="1"/>
-    <col min="11" max="11" width="14.1640625" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="14.1640625" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="19.6640625" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1">
+      <c r="A1" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="19" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-    </row>
-    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-    </row>
-    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="20"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="20"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
@@ -2593,43 +2565,43 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+    <row r="6" ht="102" customHeight="1">
+      <c r="A6" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="I6" s="17" t="s">
+      <c r="I6" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="J6" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="14" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="323" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+    <row r="7" ht="323" customHeight="1">
+      <c r="A7" s="21" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="13" t="s">
@@ -2656,13 +2628,13 @@
       <c r="I7" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="K7" s="17"/>
-    </row>
-    <row r="8" spans="1:11" ht="34" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="K7" s="14"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="20" t="s">
         <v>37</v>
       </c>
       <c r="B8" s="23" t="s">
@@ -2692,38 +2664,38 @@
       <c r="J8" s="23"/>
       <c r="K8" s="23"/>
     </row>
-    <row r="9" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="H9" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="I9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-    </row>
-    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -2736,29 +2708,29 @@
       <c r="J10" s="13"/>
       <c r="K10" s="13"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
+    <row r="15">
+      <c r="A15" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="18" t="s">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="18"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18">
       <c r="A18" s="22" t="s">
         <v>15</v>
       </c>
@@ -2772,159 +2744,162 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19" s="22" t="s">
         <v>146</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="D19" s="22">
+      <c r="D19" s="22" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20">
       <c r="A20" s="22" t="s">
         <v>146</v>
       </c>
       <c r="B20" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="22" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" s="22" t="s">
         <v>146</v>
       </c>
       <c r="B21" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="22" t="n">
         <v>35</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="22" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" s="22" t="s">
         <v>146</v>
       </c>
       <c r="B22" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="22" t="n">
         <v>45</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="22" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="18" t="s">
+    <row r="24">
+      <c r="A24" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="B24" s="18"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="18" t="s">
+      <c r="B24" s="15"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="20" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1">
+      <c r="A1" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-    </row>
-    <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="19" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-    </row>
-    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="20"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="20"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
@@ -2934,113 +2909,113 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+    <row r="6" ht="68" customHeight="1">
+      <c r="A6" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="24" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="136" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+    <row r="7" ht="136" customHeight="1">
+      <c r="A7" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="26" t="s">
         <v>156</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="E7" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="G7" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="26" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="153" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+    <row r="8" ht="153" customHeight="1">
+      <c r="A8" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-    </row>
-    <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+    </row>
+    <row r="9" ht="51" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17" t="s">
+      <c r="D9" s="14"/>
+      <c r="E9" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17" t="s">
+      <c r="G9" s="14"/>
+      <c r="H9" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="I9" s="17"/>
-    </row>
-    <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="I9" s="14"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -3051,12 +3026,13 @@
       <c r="H10" s="13"/>
       <c r="I10" s="13"/>
     </row>
-    <row r="13" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="B13" s="17" t="s">
+    <row r="13" ht="68" customHeight="1">
+      <c r="B13" s="14" t="s">
         <v>181</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>